<commit_message>
Hasil uji bench, catu LCD 5 V + level shifter, PCB hgd-v1, housing elektronik
- Catatan proyek v44: hasil uji 15 Okt. 2026, keputusan catu LCD, BOM level shifter, risiko R11/R12/R15
- Desain PCB v2: R1 220 ohm, rail +5V, soket di sisi bawah, netlist hgd-v1, usulan penempatan v2 dan gambar SVG
- Alur program v3: U4, U5, U7, U8 sebagian, E1 (sigma 38,2 counts; ambang onset 1,0 kg), data A5 dan A12
- Housing elektronik v2 dengan parameter Fusion dan kompensasi susut
- Tabel pengukuran LCD dan HX711, DS-LLS1, sketsa uji_bench_hgd

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Z5tJC56ToSqz8r7EkyAzt
</commit_message>
<xml_diff>
--- a/pcb/pcb_netlist.xlsx
+++ b/pcb/pcb_netlist.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -501,41 +501,41 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BTN</t>
+          <t>+3V3</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Tombol, GPIO25 (pull-up internal, interrupt)</t>
+          <t>Rail logika 3,3 V dari regulator papan ESP32 (KiCad: Net-(J1-VCC))</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>J1.8 (GPIO25), SW1.4</t>
+          <t>U2.1 (3V3), J1.4, J3.3 (LV), C1.1, C2.+</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LED_DRV</t>
+          <t>+5V</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Keluaran GPIO27 ke resistor</t>
+          <t>Rail 5 V dari VIN (USB) untuk LCD dan sisi HV shifter (KiCad: Net-(J2-VCC))</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>J1.10 (GPIO27), R1.1</t>
+          <t>U2.30 (VIN), J2.2, J4.3 (HV), C3.+, C4.1</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -546,32 +546,32 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ground bersama (pour tembaga sisi bawah)</t>
+          <t>Ground bersama (pour tembaga)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>J1.14 (GND), J2.14 (GND), SW1.1, D1.K, J3.1, J4.1, C1.2, C2.-, TP1.2</t>
+          <t>U2.2, U2.29, J1.1, J2.1, J3.4, J4.4, SW1.2, D1.K, C1.2, C2.-, C3.-, C4.2</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>I2C_SCL</t>
+          <t>HX_DT</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>LCD SCL, GPIO22</t>
+          <t>HX711 DOUT, GPIO18 (KiCad: Net-(J1-DT))</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>J2.2 (GPIO22), J4.4</t>
+          <t>U2.9 (GPIO18), J1.2</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -581,17 +581,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>I2C_SDA</t>
+          <t>HX_SCK</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>LCD SDA, GPIO21</t>
+          <t>HX711 SCK, GPIO19 (KiCad: Net-(J1-SCK))</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>J2.5 (GPIO21), J4.3</t>
+          <t>U2.10 (GPIO19), J1.3</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -601,17 +601,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HX_SCK</t>
+          <t>SDA_3V3</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>HX711 SCK, GPIO19</t>
+          <t>I2C SDA sisi ESP32, GPIO21 (KiCad: Net-(J3-LV1))</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>J2.6 (GPIO19), J3.3</t>
+          <t>U2.11 (GPIO21), J3.1 (LV1)</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -621,17 +621,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HX_DT</t>
+          <t>SCL_3V3</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>HX711 DOUT, GPIO18</t>
+          <t>I2C SCL sisi ESP32, GPIO22 (KiCad: Net-(J3-LV2))</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>J2.7 (GPIO18), J3.2</t>
+          <t>U2.14 (GPIO22), J3.2 (LV2)</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -641,37 +641,37 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>+3V3</t>
+          <t>SDA_5V</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Rail logika 3,3 V dari regulator papan ESP32</t>
+          <t>I2C SDA sisi LCD (KiCad: Net-(J2-SDA))</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>J2.15 (3V3), J3.4, J4.2, C1.1, C2.+, TP1.1</t>
+          <t>J4.1 (HV1), J2.3</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>LED_A</t>
+          <t>SCL_5V</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Resistor ke anoda LED</t>
+          <t>I2C SCL sisi LCD (KiCad: Net-(J2-SCL))</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>R1.2, D1.A</t>
+          <t>J4.2 (HV2), J2.4</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
@@ -681,21 +681,88 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>BTN</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tombol, GPIO25 (pull-up internal, interrupt) (KiCad: Net-(U2-D25))</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>U2.23 (GPIO25), SW1.1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>LED_DRV</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Keluaran GPIO27 ke resistor (KiCad: Net-(U2-D27))</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>U2.25 (GPIO27), R1.1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>LED_A</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Resistor ke anoda LED (KiCad: Net-(D1-A))</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>R1.2, D1.A</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>(tidak dipakai)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>VIN (J1.15) dibiarkan terbuka: papan dicatu dari USB</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>J1.15 (VIN)</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>1</v>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Kanal 3-4 level shifter</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>J3.5, J3.6, J4.5, J4.6</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Netlist dari skema KiCad hgd-v1, diperiksa 15 Okt. 2026 (kedua GND U2.2 dan U2.29 ikut). Nomor pin U2 = nomor pin header DevKit (1 = 3V3, 15 = D23, 16 = EN, 30 = VIN).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -709,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -773,27 +840,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Soket betina 1x15, pitch 2,54</t>
+          <t>ESP32 DevKit V1 30 pin</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Female pin socket 1x15, pitch 2,54 mm (generik; tanpa datasheet)</t>
+          <t>Papan: DOIT ESP32 DevKit V1; modul: ESP32-WROOM-32D (Espressif)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Connector_Generic:Conn_01x15</t>
+          <t>ESP32-DEVKIT-V1 (SnapEDA)</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Connector_PinSocket_2.54mm:PinSocket_1x15_P2.54mm_Vertical</t>
+          <t>ESP32-DEVKIT-V1:MODULE_ESP32_DEVKIT_V1 (SnapEDA, oleh "Do it")</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
@@ -801,79 +868,81 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Header kiri DevKit V1 (EN ... VIN). Baris atas PCB (y=0)</t>
+          <t>Mikrokontroler; dicolok ke dua soket betina 1x15 di sisi bawah PCB</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Standar; lubang bor 1,0 mm, pad 1,7 mm</t>
+          <t>Pitch 2,54, jarak baris 25,4, bor 1,02 mm, pad 1 = 3V3, pad 16 = EN (diperiksa). Empat lubang NPTH bawaan footprint dihapus</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>DS-CON1 (opsional); DS-ESP2</t>
+          <t>DS-ESP1, DS-ESP2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Soket betina 1x15, pitch 2,54</t>
+          <t>Soket betina 1x15 (2 pcs)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Female pin socket 1x15, pitch 2,54 mm (generik; tanpa datasheet)</t>
+          <t>Female pin socket 1x15, pitch 2,54 mm (generik)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Connector_Generic:Conn_01x15</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Connector_PinSocket_2.54mm:PinSocket_1x15_P2.54mm_Vertical</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>1</v>
+          <t>Disolder pada pad U2</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Header kanan DevKit V1 (GPIO23 ... 3V3). Baris bawah (y=25,4)</t>
+          <t>Dudukan DevKit</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Jarak antar baris J1-J2 = 25,4 mm (ukur 25,3)</t>
+          <t>Bukan footprint terpisah: hapus dua REF** PinSocket_1x15 yang menumpuk di pad U2</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>DS-CON1 (opsional); DS-ESP2</t>
+          <t>DS-CON1 (opsional)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Header pin jantan 1x4, 2,54</t>
+          <t>Soket betina 1x4</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Pin header 1x4, pitch 2,54 mm (generik; tanpa datasheet)</t>
+          <t>Female pin socket 1x4, pitch 2,54 mm (generik)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -883,7 +952,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Connector_PinHeader_2.54mm:PinHeader_1x04_P2.54mm_Vertical</t>
+          <t>Connector_PinSocket_2.54mm:PinSocket_1x04_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="F4" s="4" t="n">
@@ -891,34 +960,34 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Ke modul HX711 (GND, DT, SCK, VCC) lewat kabel jumper</t>
+          <t>Modul HX711 dicolok langsung (GND, DT, SCK, VCC)</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Urutan pin modul XFW-HX711 belum dicek; kabel jumper mengatasinya</t>
+          <t>Sisi bawah; cocokkan urutan dengan silkscreen XFW-HX711</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>DS-CON1 (opsional); DS-HX1</t>
+          <t>DS-HX1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Header pin jantan 1x4, 2,54</t>
+          <t>Soket betina 1x4</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Pin header 1x4, pitch 2,54 mm (generik; tanpa datasheet)</t>
+          <t>Female pin socket 1x4, pitch 2,54 mm (generik)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -928,7 +997,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Connector_PinHeader_2.54mm:PinHeader_1x04_P2.54mm_Vertical</t>
+          <t>Connector_PinSocket_2.54mm:PinSocket_1x04_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
@@ -936,44 +1005,44 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Ke backpack I2C LCD (GND, VCC, SDA, SCL) lewat kabel jumper</t>
+          <t>Backpack LCD lewat kabel F-M (GND, VCC 5 V, SDA, SCL)</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Urutan backpack umum GND-VCC-SDA-SCL; cek saat barang tiba</t>
+          <t>Sisi bawah</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>DS-CON1 (opsional); DS-I2C1</t>
+          <t>DS-LCD1, DS-I2C1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Tombol tactile 6x6 mm</t>
+          <t>Soket betina 1x6</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Tactile push button 6 x 6 mm, THT (generik; DS-BTN1 belum ada)</t>
+          <t>Female pin socket 1x6, pitch 2,54 mm (generik)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Switch:SW_Push</t>
+          <t>Connector_Generic:Conn_01x06</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Button_Switch_THT:SW_PUSH_6mm</t>
+          <t>Connector_PinSocket_2.54mm:PinSocket_1x06_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="F6" s="4" t="n">
@@ -981,44 +1050,44 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Tombol tunggal (START/NEXT/RESTART), GPIO25</t>
+          <t>Level shifter sisi LV (LV1, LV2, LV, GND, LV3, LV4)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Footprint sementara; hanya dua kaki diagonal dipakai. Ganti sesuai DS-BTN1</t>
+          <t>Sisi bawah; soket tidak berkunci: tandai pin 1 dan "LV"</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>DS-BTN1 (belum diambil)</t>
+          <t>DS-LLS1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>LED 5 mm</t>
+          <t>Soket betina 1x6</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>LED 5 mm diffused, THT (generik; DS-LED1 belum ada)</t>
+          <t>Female pin socket 1x6, pitch 2,54 mm (generik)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Device:LED</t>
+          <t>Connector_Generic:Conn_01x06</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>LED_THT:LED_D5.0mm</t>
+          <t>Connector_PinSocket_2.54mm:PinSocket_1x06_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="F7" s="4" t="n">
@@ -1026,44 +1095,44 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Indikator genggam, GPIO27</t>
+          <t>Level shifter sisi HV (HV1, HV2, HV, GND, HV3, HV4)</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Warna dan Vf belum diketahui</t>
+          <t>Jarak J3-J4 10,16 mm (perkiraan; ukur modul)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>DS-LED1 (belum diambil)</t>
+          <t>DS-LLS1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Resistor 100 ohm</t>
+          <t>Tombol tactile 6x6 mm, batang 13 mm</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Resistor 100 ohm, axial, 1/4 W (generik; DS-RES1 opsional)</t>
+          <t>Tactile push button 6 x 6 mm, THT, tinggi 13 mm (generik)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Switch:SW_Push</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
+          <t>Button_Switch_THT:SW_PUSH_6mm_H13mm</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
@@ -1071,44 +1140,44 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Pembatas arus LED</t>
+          <t>Tombol tunggal (START/NEXT/RESTART), GPIO25</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Dipilih untuk sekitar 13 mA dengan Vf 2,0 V (anggaran daya mencatat 15 mA); cek Vf LED</t>
+          <t>Sisi atas; menembus tutup</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>DS-RES1 (opsional)</t>
+          <t>DS-BTN1 (belum diambil)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Kapasitor keramik 100 nF</t>
+          <t>LED 5 mm</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ceramic capacitor 100 nF (generik; DS-CAP1 opsional)</t>
+          <t>LED 5 mm diffused, THT (generik)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Device:C</t>
+          <t>Device:LED</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Capacitor_THT:C_Disc_D5.0mm_W2.5mm_P5.00mm</t>
+          <t>LED_THT:LED_D5.0mm</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
@@ -1116,44 +1185,44 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Decoupling dekat J3 (catu HX711)</t>
+          <t>Indikator genggam, GPIO27</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Opsional; dari komponen lab</t>
+          <t>Sisi atas</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>DS-CAP1 (opsional)</t>
+          <t>DS-LED1 (belum diambil)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Kapasitor elektrolit 10 uF, 6,3 V atau lebih</t>
+          <t>Resistor 220 ohm</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Aluminium electrolytic capacitor 10 uF (generik; DS-CAP1 opsional)</t>
+          <t>Resistor 220 ohm, axial, 1/4 W (generik)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Device:C_Polarized</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Capacitor_THT:CP_Radial_D5.0mm_P2.00mm</t>
+          <t>Resistor_THT:R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
@@ -1161,44 +1230,44 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Decoupling dekat J3</t>
+          <t>Pembatas arus LED</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Opsional; perhatikan polaritas (+ ke 3V3)</t>
+          <t>Sekitar 6 mA pada Vf 2,0 V; sisi atas</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>DS-CAP1 (opsional)</t>
+          <t>DS-RES1 (opsional)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>TP1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Header pin jantan 1x2</t>
+          <t>Kapasitor keramik 100 nF</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Pin header 1x2, pitch 2,54 mm (generik)</t>
+          <t>Ceramic capacitor 100 nF (generik)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Connector_Generic:Conn_01x02</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Connector_PinHeader_2.54mm:PinHeader_1x02_P2.54mm_Vertical</t>
+          <t>Capacitor_THT:C_Disc_D7.0mm_W2.5mm_P5.00mm</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
@@ -1206,69 +1275,206 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Titik uji 3V3 dan GND untuk multimeter</t>
+          <t>Decoupling +3V3 dekat J1 (HX711)</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Opsional</t>
+          <t>Sisi bawah; komponen lab</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DS-CAP1 (opsional)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Kapasitor elektrolit 10 uF</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Aluminium electrolytic capacitor 10 uF, 6,3 V atau lebih (generik)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Device:C_Polarized</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Capacitor_THT:CP_Radial_D5.0mm_P2.50mm</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Bulk +3V3 dekat J1</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Sisi bawah; + ke 3V3</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>DS-CAP1 (opsional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Kapasitor elektrolit 10 uF</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Aluminium electrolytic capacitor 10 uF, 6,3 V atau lebih (generik)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Device:C_Polarized</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Capacitor_THT:CP_Radial_D5.0mm_P2.50mm</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Bulk +5V dekat J2 (LCD)</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Sisi bawah; + ke 5V</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>DS-CAP1 (opsional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Kapasitor keramik 100 nF</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Ceramic capacitor 100 nF (generik)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Device:C</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Capacitor_THT:C_Disc_D7.0mm_W2.5mm_P5.00mm</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Decoupling +5V dekat J2</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Sisi bawah</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>DS-CAP1 (opsional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>H1-H4</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Lubang M3, 3,2 mm</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Mounting hole M3 (lubang 3,2 mm)</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Lubang M3</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Mounting hole M3</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Mechanical:MountingHole</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>MountingHole:MountingHole_3.2mm_M3</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Pemasangan ke housing</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Posisi (3,-11), (43,-11), (3,44), (43,44)</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Posisi ditentukan setelah sisi atas; satu dekat SW1</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Nama simbol dan footprint di atas adalah nama pustaka standar KiCad (kolom "Pustaka:Nama") yang paling dekat dengan komponen; cocokkan dengan yang benar-benar terpasang di skema Anda dan ubah bila beda. Nama part resmi hanya ada bila komponen punya datasheet (kode DS-* di datasheet/datasheet-library.md); komponen generik ditulis sebagai deskripsi baku.</t>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Simbol dan footprint sesuai skema KiCad hgd-v1 (15 Okt. 2026). Kredit footprint U2: SnapEDA, "ESP32-DEVKIT-V1" oleh "Do it".</t>
         </is>
       </c>
     </row>
@@ -1356,22 +1562,22 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Tidak dipakai; papan diwakili J1 dan J2. Simbol kustom opsional: HGD:ESP32_DevKit_V1_30pin (belum dibuat)</t>
+          <t>U2 (SnapEDA)</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Tidak dipakai; papan diwakili J1 dan J2. Footprint kustom opsional: HGD:ESP32_DevKit_V1_Outline (belum dibuat; memuat area antena bebas tembaga)</t>
+          <t>U2 (SnapEDA)</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>J1 + J2 (soket betina 1x15)</t>
+          <t>Dua soket betina 1x15 (pad U2)</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Papan dicolok ke soket, tidak disolder</t>
+          <t>Dicolok, sisi bawah PCB</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -1398,22 +1604,22 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Tidak dipakai; modul diwakili J3. Simbol kustom opsional: HGD:HX711_Module_XFW (belum dibuat)</t>
+          <t>Diwakili J1</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Tidak dipakai (modul di luar PCB, lewat kabel jumper)</t>
+          <t>Diwakili J1</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>J3 (header 1x4: GND, DT, SCK, VCC)</t>
+          <t>J1, dicolok langsung</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Urutan pin modul belum dicek</t>
+          <t>24 x 15,6 mm terukur; header 4 pin di tengah sisi pendek; modul menggantung ke luar ke arah area LCD</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -1440,22 +1646,22 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Tidak dipakai; LCD dan backpack diwakili J4</t>
+          <t>Diwakili J2</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Tidak dipakai (di luar PCB)</t>
+          <t>Di luar PCB (dibaut ke tutup)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>J4 (header 1x4: GND, VCC, SDA, SCL), lewat backpack</t>
+          <t>J2 lewat kabel F-M</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Catu LCD 3,3 V atau 5 V masih terbuka</t>
+          <t>Catu 5 V (diputuskan 15 Okt. 2026)</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -1477,7 +1683,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>PCF8574 atau PCF8574A (NXP); penandaan chip belum diperiksa</t>
+          <t>PCF8574T (NXP), alamat 0x27</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1492,12 +1698,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Alamat 0x27 atau 0x3F menurut catatan</t>
+          <t>Pull-up SDA/SCL ke VCC: 4,93 V terukur</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1509,49 +1715,91 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
+          <t>MOD-LLS</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Level shifter 4 kanal</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Modul penggeser level dua arah 4 kanal, MOSFET BSS138 (generik)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Diwakili J3 dan J4</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Diwakili J3 dan J4</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>J3 (LV) dan J4 (HV)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Dibeli, belum tiba; ±13,3 x 16 mm; kanal 1-2 untuk SDA/SCL</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>DS-LLS1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
           <t>MOD-LC</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Load cell 80 kg</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>CZL601 (Eagle Weigh, seri CZL 601) / CZL-601 (GJ Impex); kapasitas 80 kg</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Tidak dipakai; terhubung ke modul HX711 lewat terminal (E+, E-, A-, A+)</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Tidak dipakai</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Tidak dipakai (di luar PCB)</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Terminal modul HX711</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Warna kabel: eksitasi = hitam dan putih, sinyal = merah dan hijau (hasil ukur, beda dari datasheet)</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>DS-LC1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Bagian di luar PCB, tercatat di sini supaya nama resminya tetap satu tempat. Simbol dan footprint kustom yang disebut di kolom D-E dikelola di pcb/kicad/README.md.</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Bagian di luar PCB, tercatat di sini supaya nama resminya tetap satu tempat.</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1597,12 +1845,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Pin DevKit simetris: 7,97 mm dari tiap ujung papan ke pin pertama dan terakhir</t>
+          <t>Jarak baris header level shifter 10,16 mm</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Belum diukur. Ukur jarak ujung USB ke pusat pin VIN/3V3 dan ujung antena ke pusat pin EN/GPIO23. Geser soket bila beda lebih dari 0,5 mm</t>
+          <t>Perkiraan: lebar modul 13,3 mm hanya cocok dengan 10,16. Ukur saat modul tiba sebelum jalur dibuat</t>
         </is>
       </c>
     </row>
@@ -1612,12 +1860,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Jarak antar baris 25,4 mm (hasil ukur 25,3 mm)</t>
+          <t>Header HX711 1,5 mm dari tepi modul</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Selisih 0,1 mm masih di dalam kelonggaran pin 0,5 mm di lubang 1,0 mm</t>
+          <t>Perkiraan; ukur</t>
         </is>
       </c>
     </row>
@@ -1627,12 +1875,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ujung USB rata dengan tepi kiri PCB; antena menjorok 5,5 mm melewati tepi kanan</t>
+          <t>Penempatan v2 dari tangkapan layar Fusion</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Konektor USB tidak menonjol (ukuran pengguna); area antena modul 6,19 mm harus bebas tembaga</t>
+          <t>Toleransi sekitar 1 mm; lihat pcb/desain-pcb-hgd.md Bagian 8.4 dan pcb/gambar/penempatan-pcb-hgd.svg</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1890,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Tinggi: bagian papan setinggi 6,6 mm di atas bibir soket</t>
+          <t>Zona antena 15 mm di samping dan depan antena</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Dari ukuran pengguna; tinggi soket belum dipilih</t>
+          <t>Dari ringkasan pedoman Espressif (NextPCB); belum dicocokkan dengan dokumen Espressif</t>
         </is>
       </c>
     </row>
@@ -1657,12 +1905,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>LCD dan HX711 dicatu dari 3V3</t>
+          <t>Edge.Cuts dan lubang M3 belum ditentukan</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Mengikuti catatan proyek. Backpack I2C punya pull-up ke VCC: jangan dicatu 5 V karena SDA dan SCL akan tertarik ke 5 V (ESP32 hanya 3,3 V). Eksitasi load cell pada catu 3,3 V lebih rendah dari 4,3 V pada 5 V; perlu dicek lewat uji</t>
+          <t>Setelah sisi atas selesai; satu M3 dekat SW1</t>
         </is>
       </c>
     </row>
@@ -1672,12 +1920,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>VIN tidak dipakai</t>
+          <t>Tanpa baterai; catu USB saja</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Papan dicatu dari USB; jangan menyambung catu luar ke VIN bersamaan dengan USB</t>
+          <t>Tidak ada catu luar ke VIN bersamaan dengan USB</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1940,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Cukup untuk draf non formal; tinjau bila diminta kelas</t>
+          <t>Cukup untuk perangkat berdaya USB</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1955,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Usul: dua lapis, GND pour di sisi bawah, jalur sinyal 0,3 mm, jalur 3V3 0,5 mm, jarak minimum 0,25 mm. Sesuaikan dengan aturan kelas dan kemampuan pabrik (DS-MFG1)</t>
+          <t>Usul: dua lapis, GND pour, sinyal 0,3 mm, rail 0,5 mm, jarak minimum 0,25 mm; sesuaikan dengan aturan kelas dan pabrik</t>
         </is>
       </c>
     </row>
@@ -1717,27 +1965,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Persyaratan tugas PCB (alat desain, ukuran maksimum, aturan) belum diketahui</t>
+          <t>Soket tidak berkunci</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Menunggu materi dari kelas</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Alokasi pin mengikuti tabel pin proyek: HX711 DT 18, SCK 19, LCD SDA 21, SCL 22, tombol 25, LED 27</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Dari alokasi pin di pcb/desain-pcb-hgd.md. Urutan header DevKit V1 dari gambar pinout yang dikirim</t>
+          <t>Shifter terbalik 180° memberi 5 V ke sisi LV dan GPIO: tandai pin 1 dan HV/LV di B.Silkscreen</t>
         </is>
       </c>
     </row>

</xml_diff>